<commit_message>
docs: record Sprint 2 test results in the requirements workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirements/SPMS_requirements.xlsx
+++ b/docs/requirements/SPMS_requirements.xlsx
@@ -28,7 +28,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -58,8 +60,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1057,9 +1060,6 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1107,9 +1107,6 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1154,12 +1151,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Pass. test_tc03_exit_closes_session: xe ra cổng OUT-1 tạo thanh toán chờ; thanh toán QR mock thành công thì phiên đỗ Closed, có giờ ra, sự kiện exited mở barrier.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Claude Code (pytest tự động)</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1207,9 +1214,6 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1254,12 +1258,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Pass (theo CR-02, giữ 10 phút thay vì 15). test_tc05_reservation_sets_slot_reserved: T1-A-05 chuyển Reserved, expires_at = 08:10 khi đặt lúc 08:00. Giao diện Driver (Edge) hiện đếm ngược từ 10:00.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Claude Code (pytest tự động)</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1304,12 +1318,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Pass (theo CR-02, kiểm tra ở phút 11 thay vì phút 16). test_tc06_reservation_expires_at_minute_11: phút 10 slot vẫn Reserved; phút 11 slot trở lại Available, đặt chỗ chuyển expired.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Claude Code (pytest tự động)</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1357,9 +1381,6 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1404,12 +1425,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Pass. test_tc08_fee_3h10m_is_40000: vào 08:00, ra 11:10, thanh toán chờ 40000 VND (giá 20000/2 giờ đầu + 10000/giờ làm tròn lên). test_fee_rounds_up_started_hours: 0/60/120/121/190 phút = 20000/20000/20000/30000/40000.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Claude Code (pytest tự động)</t>
+        </is>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1454,12 +1485,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Pass. test_tc09_failed_qr_keeps_barrier_closed: giao dịch QR thất bại tạo sự kiện payment_failed, barrier_opened_at rỗng, phiên đỗ vẫn Active. Giao diện Gate (Edge) hiện 'QR payment failed' và barrier Đóng.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Claude Code (pytest tự động)</t>
+        </is>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1507,9 +1548,6 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1554,12 +1592,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Pass. test_tc11_new_price_applies_to_new_sessions_only và test_tc11_fee_uses_price_at_entry: đổi per_hour 10000 sang 15000 giữa hai phiên; phiên cũ trả 40000, phiên mới trả 50000.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Claude Code (pytest tự động)</t>
+        </is>
+      </c>
+      <c r="L12" s="1" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1604,12 +1652,22 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Pass. test_tc12_report_total_equals_paid_sessions: 5 phiên Paid ngày 2026-10-19 (20000+30000+40000+20000+50000) báo cáo ra đúng tổng 160000; thanh toán lúc 00:05 ngày sau và thanh toán đang chờ không được tính. test_report_day_boundary_is_utc_plus_7 kiểm tra ranh giới ngày UTC+7.</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Claude Code (pytest tự động)</t>
+        </is>
+      </c>
+      <c r="L13" s="1" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1654,12 +1712,22 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Pass. test_tc13_driver_gets_403_on_admin_page (GET /api/audit-log) và test_tc13_driver_gets_403_on_price_admin (GET và POST /api/prices): tài khoản driver nhận HTTP 403. Giao diện: driver chỉ thấy tab Driver.</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Claude Code (pytest tự động)</t>
+        </is>
+      </c>
+      <c r="L14" s="1" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1707,9 +1775,6 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1757,9 +1822,6 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1807,9 +1869,6 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1854,12 +1913,22 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Pass. mocks/perf_tc17.py, 100 sự kiện vào liên tiếp: mean 10.0 ms, p95 11.8 ms, max 95.1 ms (giới hạn 3000 ms). Máy Intel Core i5-12500H, 15.7 GB RAM, Windows 11, SQLite. Chi tiết: docs/testing/tc17-results.md. Chỉ đo phần mềm; barrier và camera là mock.</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Claude Code (pytest tự động)</t>
+        </is>
+      </c>
+      <c r="L18" s="1" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1907,9 +1976,6 @@
           <t>Not Run</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3481,7 +3547,6 @@
       <c r="K5" t="n">
         <v>3</v>
       </c>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>SP-2;slots</t>
@@ -3932,7 +3997,6 @@
       <c r="K12" t="n">
         <v>2</v>
       </c>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>SP-4;admin</t>
@@ -4058,7 +4122,6 @@
       <c r="K14" t="n">
         <v>3</v>
       </c>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>SP-4;security</t>
@@ -4184,7 +4247,6 @@
       <c r="K16" t="n">
         <v>2</v>
       </c>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>interface;lpr</t>
@@ -5115,7 +5177,6 @@
       <c r="J2" t="n">
         <v>8</v>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">

</xml_diff>

<commit_message>
docs: record Sprint 1 test results, store dates as text
Fill TC-01, 02, 04, 14, 15 and 16 from their passing automated tests,
set executed_by to the team member, and write executed_date as ISO text
like the rest of the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QtdibwW2aJvtzsPHirJFqF
</commit_message>
<xml_diff>
--- a/docs/requirements/SPMS_requirements.xlsx
+++ b/docs/requirements/SPMS_requirements.xlsx
@@ -1057,7 +1057,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Pass. test_tc01_entry_creates_active_session: sự kiện LPR biển 30A-123.45 ở IN-1 tạo đúng 1 phiên Active với giờ vào bằng timestamp của sự kiện.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1119,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Pass. test_tc02_barrier_opens_within_3s: barrier_opened_at - received_at &lt;= 3 giây (đo thực tế p95 11,8 ms ở TC-17).</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1161,11 +1191,13 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Claude Code (pytest tự động)</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="n">
-        <v>46312</v>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1211,7 +1243,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Pass. test_tc04_free_count_matches_sensor: tầng 1 có 20 slot trống, cảm biến báo 1 slot có xe, màn hình chỗ trống hiện 19.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1268,11 +1315,13 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Claude Code (pytest tự động)</t>
-        </is>
-      </c>
-      <c r="L6" s="1" t="n">
-        <v>46312</v>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1328,11 +1377,13 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Claude Code (pytest tự động)</t>
-        </is>
-      </c>
-      <c r="L7" s="1" t="n">
-        <v>46312</v>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1435,11 +1486,13 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Claude Code (pytest tự động)</t>
-        </is>
-      </c>
-      <c r="L9" s="1" t="n">
-        <v>46312</v>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L9" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1495,11 +1548,13 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Claude Code (pytest tự động)</t>
-        </is>
-      </c>
-      <c r="L10" s="1" t="n">
-        <v>46312</v>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L10" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1602,11 +1657,13 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Claude Code (pytest tự động)</t>
-        </is>
-      </c>
-      <c r="L12" s="1" t="n">
-        <v>46312</v>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L12" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1662,11 +1719,13 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Claude Code (pytest tự động)</t>
-        </is>
-      </c>
-      <c r="L13" s="1" t="n">
-        <v>46312</v>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L13" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1722,11 +1781,13 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Claude Code (pytest tự động)</t>
-        </is>
-      </c>
-      <c r="L14" s="1" t="n">
-        <v>46312</v>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L14" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1772,7 +1833,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Pass. test_tc14_manual_open_writes_one_log: Attendant mở barrier thủ công với lý do 'Khách trả tiền mặt', audit log có đúng 1 dòng gồm người làm, giờ, lý do.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1895,22 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Pass. test_tc15_lpr_event_valid_returns_201: POST /api/lpr-events với JSON hợp lệ trả HTTP 201 và có 1 sự kiện cổng mới.</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1866,7 +1957,22 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Pass. test_tc16_low_confidence_then_manual_entry: confidence 0.6 cho action manual_required; Attendant nhập tay tạo phiên Active và 1 dòng audit log.</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1923,11 +2029,13 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Claude Code (pytest tự động)</t>
-        </is>
-      </c>
-      <c r="L18" s="1" t="n">
-        <v>46312</v>
+          <t>VUDUYLINH</t>
+        </is>
+      </c>
+      <c r="L18" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
       </c>
     </row>
     <row r="19">

</xml_diff>